<commit_message>
Made recommendation based on analysis and updated rankings chart
</commit_message>
<xml_diff>
--- a/Carrillo-Valencia_Territory_Chart.xlsx
+++ b/Carrillo-Valencia_Territory_Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brandon\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D980740-9D41-440A-B382-F0F30A6B7213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4120747-0846-404C-9080-ED9082A46033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="525" yWindow="2970" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{F64D7631-7399-4B5F-A614-76CA3BA49898}"/>
+    <workbookView xWindow="2040" yWindow="4650" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{F64D7631-7399-4B5F-A614-76CA3BA49898}"/>
   </bookViews>
   <sheets>
     <sheet name="Carrillo-Valencia_Territory_Cha" sheetId="1" r:id="rId1"/>
@@ -3107,16 +3107,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>238125</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>119063</xdr:rowOff>
+      <xdr:rowOff>80963</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3269,7 +3269,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{44998491-5EC7-48A1-BE0D-E51E51839ADF}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{44998491-5EC7-48A1-BE0D-E51E51839ADF}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="18">
   <location ref="F2:G25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0">

</xml_diff>